<commit_message>
se actualizo con los nuevos lote nuevo usariom isaaacr incluos informaicon de produccion 2026-wk33
</commit_message>
<xml_diff>
--- a/LABORES AGRICOLAS/LOTESH.xlsx
+++ b/LABORES AGRICOLAS/LOTESH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PEDRO\Produccion-Lamiformi\cv-20250714T161904Z-1-001\cv\2025\SISBANLAM2025\Merejildo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C73E0372-C7AF-46E2-9B75-F0472FBEEA2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37AD431C-5D0F-4F97-9D5C-3A878800093C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="11">
   <si>
     <t>SECTOR</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>SAN HUMBERTO</t>
+  </si>
+  <si>
+    <t>ISAAC ZAPATA</t>
   </si>
 </sst>
 </file>
@@ -593,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="20.140625" customWidth="1"/>
@@ -866,7 +869,7 @@
         <v>10.11</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E16" t="s">
         <v>9</v>
@@ -883,7 +886,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E17" t="s">
         <v>9</v>
@@ -917,7 +920,7 @@
         <v>10.25</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -934,7 +937,7 @@
         <v>10</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
@@ -951,7 +954,7 @@
         <v>10.31</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
@@ -968,7 +971,7 @@
         <v>10</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
@@ -985,7 +988,7 @@
         <v>10</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1138,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32" t="s">
         <v>9</v>
@@ -1155,9 +1158,43 @@
         <v>10</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="15">
+        <v>4</v>
+      </c>
+      <c r="B34" s="5">
+        <v>33</v>
+      </c>
+      <c r="C34" s="14">
+        <v>10</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="15">
+        <v>4</v>
+      </c>
+      <c r="B35" s="5">
+        <v>34</v>
+      </c>
+      <c r="C35" s="14">
+        <v>10</v>
+      </c>
+      <c r="D35" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E35" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>